<commit_message>
📊 Weekly RSI Screener Report – 2026-04-25
</commit_message>
<xml_diff>
--- a/docs/NSE500_stocks.xlsx
+++ b/docs/NSE500_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -576,7 +576,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LLOYDSME</t>
+          <t>POWERINDIA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1695.6</v>
+        <v>32200</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>82.2</v>
+        <v>82.68000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>70.43000000000001</v>
+        <v>77.87</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>67.43000000000001</v>
+        <v>76.13</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>26.72</v>
+        <v>23.44</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1310.68</v>
+        <v>22091.2</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1296.87</v>
+        <v>21073.92</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>740846</v>
+        <v>150269</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>95387</v>
+        <v>143523</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DATAPATTNS</t>
+          <t>LLOYDSME</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>4077.7</v>
+        <v>1695.6</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>75.44</v>
+        <v>82.2</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>71.39</v>
+        <v>70.43000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>68.44</v>
+        <v>67.43000000000001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>45.73</v>
+        <v>26.72</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>2942.89</v>
+        <v>1310.68</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>2871.7</v>
+        <v>1296.87</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1246283</v>
+        <v>740846</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>22829</v>
+        <v>95387</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GRANULES</t>
+          <t>SCHNEIDER</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>689.45</v>
+        <v>1180.1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>73.44</v>
+        <v>78.02</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>71.27</v>
+        <v>77.31</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>66.75</v>
+        <v>67.7</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>27.18</v>
+        <v>31.06</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>580.5700000000001</v>
+        <v>840.13</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>570.1900000000001</v>
+        <v>825.38</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1101438</v>
+        <v>149340</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>17084</v>
+        <v>28217</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>DATAPATTNS</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,37 +702,37 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>7328.5</v>
+        <v>4077.7</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>69.58</v>
+        <v>75.44</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>77.05</v>
+        <v>71.39</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>65.73999999999999</v>
+        <v>68.44</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>24.06</v>
+        <v>45.73</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>5827.47</v>
+        <v>2942.89</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5787.22</v>
+        <v>2871.7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>469156</v>
+        <v>1246283</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>155297</v>
+        <v>22829</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ANANDRATHI</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -741,37 +741,37 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3580.9</v>
+        <v>689.45</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>68.36</v>
+        <v>73.44</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>69.33</v>
+        <v>71.27</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>76.52</v>
+        <v>66.75</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>45.3</v>
+        <v>27.18</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3019.56</v>
+        <v>580.5700000000001</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>2914.15</v>
+        <v>570.1900000000001</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>272615</v>
+        <v>1101438</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>29729</v>
+        <v>17084</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>SAIL</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -780,37 +780,37 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1048.35</v>
+        <v>178.46</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>68.18000000000001</v>
+        <v>70.91</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>69.01000000000001</v>
+        <v>68.38</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>71.98</v>
+        <v>68.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>26.68</v>
+        <v>28.99</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>879.58</v>
+        <v>147.99</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>850.54</v>
+        <v>144.42</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>6768928</v>
+        <v>24099940</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>234427</v>
+        <v>73713</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -819,37 +819,37 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1413.8</v>
+        <v>7328.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>66.92</v>
+        <v>69.58</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>72.93000000000001</v>
+        <v>77.05</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>64</v>
+        <v>65.73999999999999</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>36.84</v>
+        <v>24.06</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>1223.82</v>
+        <v>5827.47</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>1211.28</v>
+        <v>5787.22</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>1699530</v>
+        <v>469156</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>82114</v>
+        <v>155297</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BSE</t>
+          <t>VTL</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -858,37 +858,37 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3446</v>
+        <v>590.05</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>66.02</v>
+        <v>68.73999999999999</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>69.33</v>
+        <v>74.01000000000001</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>74.37</v>
+        <v>67.11</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>28.48</v>
+        <v>28.32</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>2772.25</v>
+        <v>487.53</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2666.52</v>
+        <v>479.19</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4545846</v>
+        <v>713190</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>139952</v>
+        <v>17069</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>ANANDRATHI</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -897,37 +897,37 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>5232</v>
+        <v>3580.9</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>64.44</v>
+        <v>68.36</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>72.06</v>
+        <v>69.33</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>72.02</v>
+        <v>76.52</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>33.86</v>
+        <v>45.3</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>4381.34</v>
+        <v>3019.56</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>4243.09</v>
+        <v>2914.15</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>886794</v>
+        <v>272615</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>145031</v>
+        <v>29729</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ABSLAMC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -936,37 +936,37 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1067.65</v>
+        <v>1048.35</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>64.22</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>72.38</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>72.01000000000001</v>
+        <v>71.98</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>39.2</v>
+        <v>26.68</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>863.61</v>
+        <v>879.58</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>841.5599999999999</v>
+        <v>850.54</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>734027</v>
+        <v>6768928</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>30865</v>
+        <v>234427</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GLENMARK</t>
+          <t>SYRMA</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -975,37 +975,37 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2299.5</v>
+        <v>969.6</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>63.3</v>
+        <v>67.27</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>65.52</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>72.03</v>
+        <v>71.56</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>54.79</v>
+        <v>21.31</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>2023.92</v>
+        <v>782.99</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>1972.92</v>
+        <v>757.96</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>700705</v>
+        <v>1493405</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>64892</v>
+        <v>18677</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ASTERDM</t>
+          <t>AUROPHARMA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1014,37 +1014,37 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>705.25</v>
+        <v>1413.8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>63.03</v>
+        <v>66.92</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>62.89</v>
+        <v>72.93000000000001</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>69.41</v>
+        <v>64</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>39.23</v>
+        <v>36.84</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>627.63</v>
+        <v>1223.82</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>614.85</v>
+        <v>1211.28</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>656246</v>
+        <v>1699530</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>36457</v>
+        <v>82114</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>KIRLOSENG</t>
+          <t>TRIVENI</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1053,37 +1053,37 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1591.1</v>
+        <v>417.55</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>62.01</v>
+        <v>66.81</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>69.31</v>
+        <v>61.85</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>71.91</v>
+        <v>57.26</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>25.38</v>
+        <v>25.9</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>1244.18</v>
+        <v>373</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>1190.76</v>
+        <v>372.92</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>395140</v>
+        <v>1149992</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>23129</v>
+        <v>9145</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GMDCLTD</t>
+          <t>NMDC</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1092,37 +1092,37 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>669.85</v>
+        <v>89.29000000000001</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>59.85</v>
+        <v>66.79000000000001</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>60.9</v>
+        <v>65.18000000000001</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>72.64</v>
+        <v>68.95999999999999</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>33.45</v>
+        <v>38.97</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>553.85</v>
+        <v>77.8</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>532.14</v>
+        <v>76.38</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>6790284</v>
+        <v>25852638</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>21301</v>
+        <v>78502</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>JINDALSTEL</t>
+          <t>BSE</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1131,37 +1131,37 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1256</v>
+        <v>3446</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>59.42</v>
+        <v>66.02</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>63.02</v>
+        <v>69.33</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>67.86</v>
+        <v>74.37</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>50.15</v>
+        <v>28.48</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>1110.14</v>
+        <v>2772.25</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>1085.59</v>
+        <v>2666.52</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>1578085</v>
+        <v>4545846</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>127797</v>
+        <v>139952</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>FEDERALBNK</t>
+          <t>MAHABANK</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1170,37 +1170,37 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>293</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>59.21</v>
+        <v>65.89</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>64.63</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>69.43000000000001</v>
+        <v>66.95</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>45.31</v>
+        <v>38.56</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>259.56</v>
+        <v>63.31</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>250.72</v>
+        <v>61.69</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>9129091</v>
+        <v>25473927</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>72194</v>
+        <v>59917</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>LAURUSLABS</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1209,37 +1209,37 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1113.45</v>
+        <v>401.85</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>58.66</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>62.47</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>69.98</v>
+        <v>68.65000000000001</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>42.42</v>
+        <v>37.43</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>985.55</v>
+        <v>355.97</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>946.61</v>
+        <v>351.69</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>1844531</v>
+        <v>13965303</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>60125</v>
+        <v>389661</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>EMCURE</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1248,37 +1248,37 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1637.2</v>
+        <v>316.4</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>58.49</v>
+        <v>65.33</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>61.04</v>
+        <v>67.02</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>63.94</v>
+        <v>62.65</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>52.14</v>
+        <v>32.46</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>1463.46</v>
+        <v>286.09</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>1436.84</v>
+        <v>284.71</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>283077</v>
+        <v>15917825</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>31040</v>
+        <v>294271</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>CUMMINSIND</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1287,37 +1287,37 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1856</v>
+        <v>5232</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>58.27</v>
+        <v>64.44</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>72.06</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>65.33</v>
+        <v>72.02</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>45</v>
+        <v>33.86</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>1558.76</v>
+        <v>4381.34</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>1506.38</v>
+        <v>4243.09</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1281281</v>
+        <v>886794</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>88733</v>
+        <v>145031</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>NATIONALUM</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1326,37 +1326,37 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>456</v>
+        <v>437.05</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>57.77</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>62.34</v>
+        <v>78.84</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>68.7</v>
+        <v>81.8</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>29.79</v>
+        <v>47.7</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>414.47</v>
+        <v>325.52</v>
       </c>
       <c r="I22" s="4" t="n">
-        <v>407.52</v>
+        <v>304.17</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>13707759</v>
+        <v>14848438</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>281020</v>
+        <v>80270</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>J&amp;KBANK</t>
+          <t>ABSLAMC</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1365,70 +1365,967 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>126.05</v>
+        <v>1067.65</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>54.55</v>
+        <v>64.22</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>63.71</v>
+        <v>72.38</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>62.79</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>36.88</v>
+        <v>39.2</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>110.57</v>
+        <v>863.61</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>108.98</v>
+        <v>841.5599999999999</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>6404834</v>
+        <v>734027</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>13880</v>
+        <v>30865</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>3824.8</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>63.82</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>60.68</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>62.62</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>3201.84</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>3086.93</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>1306546</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>21779</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>GLENMARK</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>2299.5</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>72.03</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>54.79</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>2023.92</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>1972.92</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>700705</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>64892</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>705.25</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>63.03</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>62.89</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>69.41</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>39.23</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>627.63</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>614.85</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>656246</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>36457</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>KIRLOSENG</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1591.1</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>62.01</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>69.31</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>71.91</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>25.38</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>1244.18</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>1190.76</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>395140</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>23129</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>783.3</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>61.23</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>64.03</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>743.8</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>734.5700000000001</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>2032258</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>101488</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>SARDAEN</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>581.4</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>60.33</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>60.29</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>64.81</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>29.59</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>521.13</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>513.1799999999999</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>661440</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>20487</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>210.07</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>65.88</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>56.11</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>186.76</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>181.88</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>31612445</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>261996</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>NATCOPHARM</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>1093.2</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>59.89</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>66.83</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>37.83</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>938.62</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>938.4299999999999</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>871521</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>19580</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GMDCLTD</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>669.85</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>72.64</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>33.45</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>553.85</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>532.14</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>6790284</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>21301</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>2760.9</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>59.47</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>70.75</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>79.95</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>52.72</v>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>2233.23</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>2105.73</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>3727743</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>70269</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>1256</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>59.42</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>63.02</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>67.86</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>50.15</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>1110.14</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>1085.59</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>1578085</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>127797</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>FEDERALBNK</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>293</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>59.21</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>64.63</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>69.43000000000001</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>45.31</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>259.56</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>250.72</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>9129091</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>72194</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>LAURUSLABS</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>1113.45</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>58.66</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>62.47</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>42.42</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>985.55</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>946.61</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>1844531</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>60125</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>EMCURE</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>1637.2</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>58.49</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>61.04</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>63.94</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>52.14</v>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>1463.46</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>1436.84</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>283077</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>31040</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>6452</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>60.24</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>70.98999999999999</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>5822.93</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>5621.84</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>165894</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>33090</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>BHARATFORG</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>1856</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>58.27</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>65.33</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>1558.76</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>1506.38</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>1281281</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>88733</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>456</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>29.79</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>414.47</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>407.52</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>13707759</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>281020</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>284.8</v>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>57.07</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>67.69</v>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>66.56</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>30.92</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>256.09</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>252.05</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>20869156</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>358286</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>1101.1</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>56.02</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>60.01</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>65.04000000000001</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>1014.15</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>984.42</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>18057938</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>1016383</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>4410</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>55.53</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>62.41</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>63.39</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>44.59</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>4015.88</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>3932.88</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>1206041</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>391187</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>J&amp;KBANK</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>126.05</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>63.71</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>62.79</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>36.88</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>110.57</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>108.98</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>6404834</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>13880</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
           <t>HINDCOPPER</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
         <v>541.5</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D45" s="4" t="n">
         <v>52.88</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E45" s="4" t="n">
         <v>60.66</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="F45" s="4" t="n">
         <v>62.74</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="G45" s="4" t="n">
         <v>67.92</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="H45" s="4" t="n">
         <v>462.08</v>
       </c>
-      <c r="I24" s="4" t="n">
+      <c r="I45" s="4" t="n">
         <v>434.28</v>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="J45" s="4" t="n">
         <v>10254865</v>
       </c>
-      <c r="K24" s="4" t="n">
+      <c r="K45" s="4" t="n">
         <v>52364</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>720.95</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>49.71</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>62.58</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>75.64</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>47.05</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>613.38</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>583.63</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>16192328</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>281517</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>LUPIN</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>2296.1</v>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>47.89</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>61.13</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>35.57</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>2172.27</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>2139.04</v>
+      </c>
+      <c r="J47" s="4" t="n">
+        <v>1063369</v>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>104973</v>
       </c>
     </row>
   </sheetData>
@@ -1456,6 +2353,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2953,7 +3873,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>GODREJIND</t>
+          <t>CLEAN</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -2962,22 +3882,22 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>990.55</v>
+        <v>816.75</v>
       </c>
       <c r="D62" s="4" t="n">
         <v>68.31</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>51.51</v>
+        <v>46.37</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>50.82</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>CLEAN</t>
+          <t>GODREJIND</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2986,16 +3906,16 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>816.75</v>
+        <v>990.55</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>68.31</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>46.37</v>
+        <v>51.51</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>37.8</v>
+        <v>50.82</v>
       </c>
     </row>
     <row r="64">
@@ -3481,7 +4401,7 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>SWSOLAR</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -3490,22 +4410,22 @@
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>401.85</v>
+        <v>213.31</v>
       </c>
       <c r="D84" s="4" t="n">
         <v>65.70999999999999</v>
       </c>
       <c r="E84" s="4" t="n">
-        <v>68.56999999999999</v>
+        <v>52.65</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>68.65000000000001</v>
+        <v>40.12</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>SWSOLAR</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -3514,16 +4434,16 @@
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>213.31</v>
+        <v>401.85</v>
       </c>
       <c r="D85" s="4" t="n">
         <v>65.70999999999999</v>
       </c>
       <c r="E85" s="4" t="n">
-        <v>52.65</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>40.12</v>
+        <v>68.65000000000001</v>
       </c>
     </row>
     <row r="86">
@@ -3625,7 +4545,7 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MANYAVAR</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -3634,22 +4554,22 @@
         </is>
       </c>
       <c r="C90" s="4" t="n">
-        <v>450.05</v>
+        <v>316.4</v>
       </c>
       <c r="D90" s="4" t="n">
         <v>65.33</v>
       </c>
       <c r="E90" s="4" t="n">
-        <v>40.61</v>
+        <v>67.02</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>30.74</v>
+        <v>62.65</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>NLCINDIA</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -3658,22 +4578,22 @@
         </is>
       </c>
       <c r="C91" s="4" t="n">
-        <v>316.4</v>
+        <v>299.1</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>65.33</v>
       </c>
       <c r="E91" s="4" t="n">
-        <v>67.02</v>
+        <v>66.7</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>62.65</v>
+        <v>65.45</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>NLCINDIA</t>
+          <t>MANYAVAR</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -3682,16 +4602,16 @@
         </is>
       </c>
       <c r="C92" s="4" t="n">
-        <v>299.1</v>
+        <v>450.05</v>
       </c>
       <c r="D92" s="4" t="n">
         <v>65.33</v>
       </c>
       <c r="E92" s="4" t="n">
-        <v>66.7</v>
+        <v>40.61</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>65.45</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="93">
@@ -4273,7 +5193,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>AIAENG</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -4282,22 +5202,22 @@
         </is>
       </c>
       <c r="C117" s="4" t="n">
-        <v>2327.3</v>
+        <v>4014.3</v>
       </c>
       <c r="D117" s="4" t="n">
         <v>63.76</v>
       </c>
       <c r="E117" s="4" t="n">
-        <v>52.51</v>
+        <v>60.6</v>
       </c>
       <c r="F117" s="4" t="n">
-        <v>49</v>
+        <v>58.2</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>AIAENG</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -4306,16 +5226,16 @@
         </is>
       </c>
       <c r="C118" s="4" t="n">
-        <v>4014.3</v>
+        <v>2327.3</v>
       </c>
       <c r="D118" s="4" t="n">
         <v>63.76</v>
       </c>
       <c r="E118" s="4" t="n">
-        <v>60.6</v>
+        <v>52.51</v>
       </c>
       <c r="F118" s="4" t="n">
-        <v>58.2</v>
+        <v>49</v>
       </c>
     </row>
     <row r="119">
@@ -4945,7 +5865,7 @@
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>VMM</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -4954,22 +5874,22 @@
         </is>
       </c>
       <c r="C145" s="4" t="n">
-        <v>1317.1</v>
+        <v>123.34</v>
       </c>
       <c r="D145" s="4" t="n">
         <v>61.94</v>
       </c>
       <c r="E145" s="4" t="n">
-        <v>57.85</v>
+        <v>51.17</v>
       </c>
       <c r="F145" s="4" t="n">
-        <v>57.55</v>
+        <v>51.54</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>VMM</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -4978,16 +5898,16 @@
         </is>
       </c>
       <c r="C146" s="4" t="n">
-        <v>123.34</v>
+        <v>1317.1</v>
       </c>
       <c r="D146" s="4" t="n">
         <v>61.94</v>
       </c>
       <c r="E146" s="4" t="n">
-        <v>51.17</v>
+        <v>57.85</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>51.54</v>
+        <v>57.55</v>
       </c>
     </row>
     <row r="147">
@@ -5569,7 +6489,7 @@
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>WELSPUNLIV</t>
+          <t>ZEEL</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -5578,22 +6498,22 @@
         </is>
       </c>
       <c r="C171" s="4" t="n">
-        <v>130.16</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="D171" s="4" t="n">
         <v>60.28</v>
       </c>
       <c r="E171" s="4" t="n">
-        <v>53.17</v>
+        <v>48.47</v>
       </c>
       <c r="F171" s="4" t="n">
-        <v>50.49</v>
+        <v>38.94</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>ZEEL</t>
+          <t>WELSPUNLIV</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -5602,16 +6522,16 @@
         </is>
       </c>
       <c r="C172" s="4" t="n">
-        <v>88.09999999999999</v>
+        <v>130.16</v>
       </c>
       <c r="D172" s="4" t="n">
         <v>60.28</v>
       </c>
       <c r="E172" s="4" t="n">
-        <v>48.47</v>
+        <v>53.17</v>
       </c>
       <c r="F172" s="4" t="n">
-        <v>38.94</v>
+        <v>50.49</v>
       </c>
     </row>
     <row r="173">
@@ -5713,7 +6633,7 @@
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>ATUL</t>
+          <t>DCMSHRIRAM</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -5722,22 +6642,22 @@
         </is>
       </c>
       <c r="C177" s="4" t="n">
-        <v>6680.5</v>
+        <v>1187.1</v>
       </c>
       <c r="D177" s="4" t="n">
         <v>60.09</v>
       </c>
       <c r="E177" s="4" t="n">
-        <v>60.3</v>
+        <v>53.84</v>
       </c>
       <c r="F177" s="4" t="n">
-        <v>50.95</v>
+        <v>53.55</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>DCMSHRIRAM</t>
+          <t>ATUL</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -5746,16 +6666,16 @@
         </is>
       </c>
       <c r="C178" s="4" t="n">
-        <v>1187.1</v>
+        <v>6680.5</v>
       </c>
       <c r="D178" s="4" t="n">
         <v>60.09</v>
       </c>
       <c r="E178" s="4" t="n">
-        <v>53.84</v>
+        <v>60.3</v>
       </c>
       <c r="F178" s="4" t="n">
-        <v>53.55</v>
+        <v>50.95</v>
       </c>
     </row>
     <row r="179">
@@ -6649,7 +7569,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>CRISIL</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="B216" s="3" t="inlineStr">
@@ -6658,22 +7578,22 @@
         </is>
       </c>
       <c r="C216" s="4" t="n">
-        <v>4269.4</v>
+        <v>1856</v>
       </c>
       <c r="D216" s="4" t="n">
         <v>58.27</v>
       </c>
       <c r="E216" s="4" t="n">
-        <v>47.38</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F216" s="4" t="n">
-        <v>48.53</v>
+        <v>65.33</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>CRISIL</t>
         </is>
       </c>
       <c r="B217" s="3" t="inlineStr">
@@ -6682,16 +7602,16 @@
         </is>
       </c>
       <c r="C217" s="4" t="n">
-        <v>1856</v>
+        <v>4269.4</v>
       </c>
       <c r="D217" s="4" t="n">
         <v>58.27</v>
       </c>
       <c r="E217" s="4" t="n">
-        <v>65.40000000000001</v>
+        <v>47.38</v>
       </c>
       <c r="F217" s="4" t="n">
-        <v>65.33</v>
+        <v>48.53</v>
       </c>
     </row>
     <row r="218">
@@ -6745,7 +7665,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>PAYTM</t>
+          <t>BALRAMCHIN</t>
         </is>
       </c>
       <c r="B220" s="3" t="inlineStr">
@@ -6754,22 +7674,22 @@
         </is>
       </c>
       <c r="C220" s="4" t="n">
-        <v>1147.35</v>
+        <v>516.1</v>
       </c>
       <c r="D220" s="4" t="n">
         <v>57.96</v>
       </c>
       <c r="E220" s="4" t="n">
-        <v>50.66</v>
+        <v>61.88</v>
       </c>
       <c r="F220" s="4" t="n">
-        <v>56.98</v>
+        <v>54.51</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>BALRAMCHIN</t>
+          <t>PAYTM</t>
         </is>
       </c>
       <c r="B221" s="3" t="inlineStr">
@@ -6778,16 +7698,16 @@
         </is>
       </c>
       <c r="C221" s="4" t="n">
-        <v>516.1</v>
+        <v>1147.35</v>
       </c>
       <c r="D221" s="4" t="n">
         <v>57.96</v>
       </c>
       <c r="E221" s="4" t="n">
-        <v>61.88</v>
+        <v>50.66</v>
       </c>
       <c r="F221" s="4" t="n">
-        <v>54.51</v>
+        <v>56.98</v>
       </c>
     </row>
     <row r="222">
@@ -6961,7 +7881,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>HONAUT</t>
+          <t>GLAXO</t>
         </is>
       </c>
       <c r="B229" s="3" t="inlineStr">
@@ -6970,22 +7890,22 @@
         </is>
       </c>
       <c r="C229" s="4" t="n">
-        <v>31365</v>
+        <v>2472</v>
       </c>
       <c r="D229" s="4" t="n">
         <v>57.58</v>
       </c>
       <c r="E229" s="4" t="n">
-        <v>47.64</v>
+        <v>48.15</v>
       </c>
       <c r="F229" s="4" t="n">
-        <v>41.42</v>
+        <v>50.71</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>GLAXO</t>
+          <t>HONAUT</t>
         </is>
       </c>
       <c r="B230" s="3" t="inlineStr">
@@ -6994,16 +7914,16 @@
         </is>
       </c>
       <c r="C230" s="4" t="n">
-        <v>2472</v>
+        <v>31365</v>
       </c>
       <c r="D230" s="4" t="n">
         <v>57.58</v>
       </c>
       <c r="E230" s="4" t="n">
-        <v>48.15</v>
+        <v>47.64</v>
       </c>
       <c r="F230" s="4" t="n">
-        <v>50.71</v>
+        <v>41.42</v>
       </c>
     </row>
     <row r="231">
@@ -7489,7 +8409,7 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>IOB</t>
         </is>
       </c>
       <c r="B251" s="3" t="inlineStr">
@@ -7498,22 +8418,22 @@
         </is>
       </c>
       <c r="C251" s="4" t="n">
-        <v>1700.1</v>
+        <v>35.01</v>
       </c>
       <c r="D251" s="4" t="n">
         <v>56.46</v>
       </c>
       <c r="E251" s="4" t="n">
-        <v>41.86</v>
+        <v>47.76</v>
       </c>
       <c r="F251" s="4" t="n">
-        <v>40.85</v>
+        <v>42.55</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>IOB</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B252" s="3" t="inlineStr">
@@ -7522,16 +8442,16 @@
         </is>
       </c>
       <c r="C252" s="4" t="n">
-        <v>35.01</v>
+        <v>1700.1</v>
       </c>
       <c r="D252" s="4" t="n">
         <v>56.46</v>
       </c>
       <c r="E252" s="4" t="n">
-        <v>47.76</v>
+        <v>41.86</v>
       </c>
       <c r="F252" s="4" t="n">
-        <v>42.55</v>
+        <v>40.85</v>
       </c>
     </row>
     <row r="253">
@@ -7657,7 +8577,7 @@
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>NSLNISP</t>
+          <t>AADHARHFC</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
@@ -7666,22 +8586,22 @@
         </is>
       </c>
       <c r="C258" s="4" t="n">
-        <v>40.96</v>
+        <v>488.1</v>
       </c>
       <c r="D258" s="4" t="n">
         <v>56.17</v>
       </c>
       <c r="E258" s="4" t="n">
-        <v>51.64</v>
+        <v>53.98</v>
       </c>
       <c r="F258" s="4" t="n">
-        <v>48.74</v>
+        <v>56.88</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>AADHARHFC</t>
+          <t>TIMKEN</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
@@ -7690,22 +8610,22 @@
         </is>
       </c>
       <c r="C259" s="4" t="n">
-        <v>488.1</v>
+        <v>3517.6</v>
       </c>
       <c r="D259" s="4" t="n">
         <v>56.17</v>
       </c>
       <c r="E259" s="4" t="n">
-        <v>53.98</v>
+        <v>61.51</v>
       </c>
       <c r="F259" s="4" t="n">
-        <v>56.88</v>
+        <v>56</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>TIMKEN</t>
+          <t>NSLNISP</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
@@ -7714,16 +8634,16 @@
         </is>
       </c>
       <c r="C260" s="4" t="n">
-        <v>3517.6</v>
+        <v>40.96</v>
       </c>
       <c r="D260" s="4" t="n">
         <v>56.17</v>
       </c>
       <c r="E260" s="4" t="n">
-        <v>61.51</v>
+        <v>51.64</v>
       </c>
       <c r="F260" s="4" t="n">
-        <v>56</v>
+        <v>48.74</v>
       </c>
     </row>
     <row r="261">
@@ -7993,7 +8913,7 @@
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>EIHOTEL</t>
+          <t>NAM-INDIA</t>
         </is>
       </c>
       <c r="B272" s="3" t="inlineStr">
@@ -8002,22 +8922,22 @@
         </is>
       </c>
       <c r="C272" s="4" t="n">
-        <v>326.4</v>
+        <v>979.35</v>
       </c>
       <c r="D272" s="4" t="n">
         <v>55.6</v>
       </c>
       <c r="E272" s="4" t="n">
-        <v>46.7</v>
+        <v>60.48</v>
       </c>
       <c r="F272" s="4" t="n">
-        <v>48.55</v>
+        <v>69.20999999999999</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>NAM-INDIA</t>
+          <t>EIHOTEL</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
@@ -8026,16 +8946,16 @@
         </is>
       </c>
       <c r="C273" s="4" t="n">
-        <v>979.35</v>
+        <v>326.4</v>
       </c>
       <c r="D273" s="4" t="n">
         <v>55.6</v>
       </c>
       <c r="E273" s="4" t="n">
-        <v>60.48</v>
+        <v>46.7</v>
       </c>
       <c r="F273" s="4" t="n">
-        <v>69.20999999999999</v>
+        <v>48.55</v>
       </c>
     </row>
     <row r="274">
@@ -9121,7 +10041,7 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>CENTRALBK</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B319" s="3" t="inlineStr">
@@ -9130,22 +10050,22 @@
         </is>
       </c>
       <c r="C319" s="4" t="n">
-        <v>36.01</v>
+        <v>999.4</v>
       </c>
       <c r="D319" s="4" t="n">
         <v>53.17</v>
       </c>
       <c r="E319" s="4" t="n">
-        <v>48.19</v>
+        <v>44.24</v>
       </c>
       <c r="F319" s="4" t="n">
-        <v>44.34</v>
+        <v>51.24</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>CENTRALBK</t>
         </is>
       </c>
       <c r="B320" s="3" t="inlineStr">
@@ -9154,16 +10074,16 @@
         </is>
       </c>
       <c r="C320" s="4" t="n">
-        <v>999.4</v>
+        <v>36.01</v>
       </c>
       <c r="D320" s="4" t="n">
         <v>53.17</v>
       </c>
       <c r="E320" s="4" t="n">
-        <v>44.24</v>
+        <v>48.19</v>
       </c>
       <c r="F320" s="4" t="n">
-        <v>51.24</v>
+        <v>44.34</v>
       </c>
     </row>
     <row r="321">
@@ -9241,7 +10161,7 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MUTHOOTFIN</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B324" s="3" t="inlineStr">
@@ -9250,22 +10170,22 @@
         </is>
       </c>
       <c r="C324" s="4" t="n">
-        <v>3493.5</v>
+        <v>34.2</v>
       </c>
       <c r="D324" s="4" t="n">
         <v>52.92</v>
       </c>
       <c r="E324" s="4" t="n">
-        <v>54.42</v>
+        <v>40.01</v>
       </c>
       <c r="F324" s="4" t="n">
-        <v>68.66</v>
+        <v>37.05</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MUTHOOTFIN</t>
         </is>
       </c>
       <c r="B325" s="3" t="inlineStr">
@@ -9274,16 +10194,16 @@
         </is>
       </c>
       <c r="C325" s="4" t="n">
-        <v>34.2</v>
+        <v>3493.5</v>
       </c>
       <c r="D325" s="4" t="n">
         <v>52.92</v>
       </c>
       <c r="E325" s="4" t="n">
-        <v>40.01</v>
+        <v>54.42</v>
       </c>
       <c r="F325" s="4" t="n">
-        <v>37.05</v>
+        <v>68.66</v>
       </c>
     </row>
     <row r="326">
@@ -9481,7 +10401,7 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>KIRLOSBROS</t>
+          <t>ESCORTS</t>
         </is>
       </c>
       <c r="B334" s="3" t="inlineStr">
@@ -9490,22 +10410,22 @@
         </is>
       </c>
       <c r="C334" s="4" t="n">
-        <v>1645</v>
+        <v>3231.3</v>
       </c>
       <c r="D334" s="4" t="n">
         <v>52.58</v>
       </c>
       <c r="E334" s="4" t="n">
-        <v>50.06</v>
+        <v>45.85</v>
       </c>
       <c r="F334" s="4" t="n">
-        <v>51.39</v>
+        <v>49.62</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>ESCORTS</t>
+          <t>KIRLOSBROS</t>
         </is>
       </c>
       <c r="B335" s="3" t="inlineStr">
@@ -9514,22 +10434,22 @@
         </is>
       </c>
       <c r="C335" s="4" t="n">
-        <v>3231.3</v>
+        <v>1645</v>
       </c>
       <c r="D335" s="4" t="n">
         <v>52.58</v>
       </c>
       <c r="E335" s="4" t="n">
-        <v>45.85</v>
+        <v>50.06</v>
       </c>
       <c r="F335" s="4" t="n">
-        <v>49.62</v>
+        <v>51.39</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>IRB</t>
+          <t>MSUMI</t>
         </is>
       </c>
       <c r="B336" s="3" t="inlineStr">
@@ -9538,22 +10458,22 @@
         </is>
       </c>
       <c r="C336" s="4" t="n">
-        <v>21.63</v>
+        <v>39.9</v>
       </c>
       <c r="D336" s="4" t="n">
         <v>52.52</v>
       </c>
       <c r="E336" s="4" t="n">
-        <v>51.67</v>
+        <v>44.11</v>
       </c>
       <c r="F336" s="4" t="n">
-        <v>47.77</v>
+        <v>48.44</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MSUMI</t>
+          <t>IRB</t>
         </is>
       </c>
       <c r="B337" s="3" t="inlineStr">
@@ -9562,16 +10482,16 @@
         </is>
       </c>
       <c r="C337" s="4" t="n">
-        <v>39.9</v>
+        <v>21.63</v>
       </c>
       <c r="D337" s="4" t="n">
         <v>52.52</v>
       </c>
       <c r="E337" s="4" t="n">
-        <v>44.11</v>
+        <v>51.67</v>
       </c>
       <c r="F337" s="4" t="n">
-        <v>48.44</v>
+        <v>47.77</v>
       </c>
     </row>
     <row r="338">
@@ -10177,7 +11097,7 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>UNOMINDA</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="B363" s="3" t="inlineStr">
@@ -10186,22 +11106,22 @@
         </is>
       </c>
       <c r="C363" s="4" t="n">
-        <v>1108.1</v>
+        <v>10815.5</v>
       </c>
       <c r="D363" s="4" t="n">
         <v>51.45</v>
       </c>
       <c r="E363" s="4" t="n">
-        <v>46.49</v>
+        <v>40.94</v>
       </c>
       <c r="F363" s="4" t="n">
-        <v>54.54</v>
+        <v>45.88</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>UNOMINDA</t>
         </is>
       </c>
       <c r="B364" s="3" t="inlineStr">
@@ -10210,16 +11130,16 @@
         </is>
       </c>
       <c r="C364" s="4" t="n">
-        <v>10815.5</v>
+        <v>1108.1</v>
       </c>
       <c r="D364" s="4" t="n">
         <v>51.45</v>
       </c>
       <c r="E364" s="4" t="n">
-        <v>40.94</v>
+        <v>46.49</v>
       </c>
       <c r="F364" s="4" t="n">
-        <v>45.88</v>
+        <v>54.54</v>
       </c>
     </row>
     <row r="365">
@@ -10681,7 +11601,7 @@
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>360ONE</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="B384" s="3" t="inlineStr">
@@ -10690,22 +11610,22 @@
         </is>
       </c>
       <c r="C384" s="4" t="n">
-        <v>1039.6</v>
+        <v>635.35</v>
       </c>
       <c r="D384" s="4" t="n">
         <v>49.8</v>
       </c>
       <c r="E384" s="4" t="n">
-        <v>47.01</v>
+        <v>43.41</v>
       </c>
       <c r="F384" s="4" t="n">
-        <v>53.95</v>
+        <v>48.38</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="B385" s="3" t="inlineStr">
@@ -10714,16 +11634,16 @@
         </is>
       </c>
       <c r="C385" s="4" t="n">
-        <v>635.35</v>
+        <v>1039.6</v>
       </c>
       <c r="D385" s="4" t="n">
         <v>49.8</v>
       </c>
       <c r="E385" s="4" t="n">
-        <v>43.41</v>
+        <v>47.01</v>
       </c>
       <c r="F385" s="4" t="n">
-        <v>48.38</v>
+        <v>53.95</v>
       </c>
     </row>
     <row r="386">
@@ -11185,7 +12105,7 @@
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>DOMS</t>
+          <t>BANKINDIA</t>
         </is>
       </c>
       <c r="B405" s="3" t="inlineStr">
@@ -11194,22 +12114,22 @@
         </is>
       </c>
       <c r="C405" s="4" t="n">
-        <v>2315.8</v>
+        <v>147.44</v>
       </c>
       <c r="D405" s="4" t="n">
         <v>47.65</v>
       </c>
       <c r="E405" s="4" t="n">
-        <v>46.19</v>
+        <v>50.85</v>
       </c>
       <c r="F405" s="4" t="n">
-        <v>50.56</v>
+        <v>58.19</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>BANKINDIA</t>
+          <t>DOMS</t>
         </is>
       </c>
       <c r="B406" s="3" t="inlineStr">
@@ -11218,16 +12138,16 @@
         </is>
       </c>
       <c r="C406" s="4" t="n">
-        <v>147.44</v>
+        <v>2315.8</v>
       </c>
       <c r="D406" s="4" t="n">
         <v>47.65</v>
       </c>
       <c r="E406" s="4" t="n">
-        <v>50.85</v>
+        <v>46.19</v>
       </c>
       <c r="F406" s="4" t="n">
-        <v>58.19</v>
+        <v>50.56</v>
       </c>
     </row>
     <row r="407">
@@ -11977,7 +12897,7 @@
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>PFIZER</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B438" s="3" t="inlineStr">
@@ -11986,22 +12906,22 @@
         </is>
       </c>
       <c r="C438" s="4" t="n">
-        <v>4733.2</v>
+        <v>370.85</v>
       </c>
       <c r="D438" s="4" t="n">
         <v>45.07</v>
       </c>
       <c r="E438" s="4" t="n">
-        <v>45.67</v>
+        <v>38.25</v>
       </c>
       <c r="F438" s="4" t="n">
-        <v>49.81</v>
+        <v>46.49</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>PFIZER</t>
         </is>
       </c>
       <c r="B439" s="3" t="inlineStr">
@@ -12010,16 +12930,16 @@
         </is>
       </c>
       <c r="C439" s="4" t="n">
-        <v>370.85</v>
+        <v>4733.2</v>
       </c>
       <c r="D439" s="4" t="n">
         <v>45.07</v>
       </c>
       <c r="E439" s="4" t="n">
-        <v>38.25</v>
+        <v>45.67</v>
       </c>
       <c r="F439" s="4" t="n">
-        <v>46.49</v>
+        <v>49.81</v>
       </c>
     </row>
     <row r="440">
@@ -12241,7 +13161,7 @@
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>MRF</t>
+          <t>CEATLTD</t>
         </is>
       </c>
       <c r="B449" s="3" t="inlineStr">
@@ -12250,22 +13170,22 @@
         </is>
       </c>
       <c r="C449" s="4" t="n">
-        <v>132145</v>
+        <v>3476.2</v>
       </c>
       <c r="D449" s="4" t="n">
         <v>44.34</v>
       </c>
       <c r="E449" s="4" t="n">
-        <v>42.88</v>
+        <v>45.16</v>
       </c>
       <c r="F449" s="4" t="n">
-        <v>50.42</v>
+        <v>55.57</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>CEATLTD</t>
+          <t>MRF</t>
         </is>
       </c>
       <c r="B450" s="3" t="inlineStr">
@@ -12274,16 +13194,16 @@
         </is>
       </c>
       <c r="C450" s="4" t="n">
-        <v>3476.2</v>
+        <v>132145</v>
       </c>
       <c r="D450" s="4" t="n">
         <v>44.34</v>
       </c>
       <c r="E450" s="4" t="n">
-        <v>45.16</v>
+        <v>42.88</v>
       </c>
       <c r="F450" s="4" t="n">
-        <v>55.57</v>
+        <v>50.42</v>
       </c>
     </row>
     <row r="451">
@@ -12625,7 +13545,7 @@
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>JUSTDIAL</t>
         </is>
       </c>
       <c r="B465" s="3" t="inlineStr">
@@ -12634,22 +13554,22 @@
         </is>
       </c>
       <c r="C465" s="4" t="n">
-        <v>1327.8</v>
+        <v>527.4</v>
       </c>
       <c r="D465" s="4" t="n">
         <v>42.69</v>
       </c>
       <c r="E465" s="4" t="n">
-        <v>39.43</v>
+        <v>32.42</v>
       </c>
       <c r="F465" s="4" t="n">
-        <v>47.61</v>
+        <v>34.79</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>JUSTDIAL</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B466" s="3" t="inlineStr">
@@ -12658,16 +13578,16 @@
         </is>
       </c>
       <c r="C466" s="4" t="n">
-        <v>527.4</v>
+        <v>1327.8</v>
       </c>
       <c r="D466" s="4" t="n">
         <v>42.69</v>
       </c>
       <c r="E466" s="4" t="n">
-        <v>32.42</v>
+        <v>39.43</v>
       </c>
       <c r="F466" s="4" t="n">
-        <v>34.79</v>
+        <v>47.61</v>
       </c>
     </row>
     <row r="467">

</xml_diff>